<commit_message>
S6(W6.4): example 资产落地——4 旧样例按 S4 分流重生成(IB 无 fabric j2) + 6 新场景导入成品(plan/para/excel/templates/meta ready)
</commit_message>
<xml_diff>
--- a/example/128H100-IB/excel/connection.xlsx
+++ b/example/128H100-IB/excel/connection.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="终端连接表-参数网" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="终端连接表-存储网" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="终端连接表-业务网" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="终端连接表-带外网" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VLAN网关表-参数网" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VLAN网关表-存储网" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VLAN网关表-业务网" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="终端连接表-参数网" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="终端连接表-存储网" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="终端连接表-业务网" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="终端连接表-带外网" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="VLAN网关表-参数网" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="VLAN网关表-存储网" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="VLAN网关表-业务网" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48,7 +48,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -56,22 +56,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -450,27 +441,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>己端设备</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>己端接口</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>己端VLAN</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>己端描述</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>备注信息</t>
         </is>
@@ -26098,27 +26089,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>己端设备</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>己端接口</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>己端VLAN</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>己端描述</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>备注信息</t>
         </is>
@@ -27746,27 +27737,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>己端设备</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>己端接口</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>己端VLAN</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>己端描述</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>备注信息</t>
         </is>
@@ -30994,27 +30985,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>己端设备</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>己端接口</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>己端VLAN</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>己端描述</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>备注信息</t>
         </is>
@@ -31441,22 +31432,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>己端设备</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>网关VLAN</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>网关IP</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>备注信息</t>
         </is>
@@ -31803,22 +31794,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>己端设备</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>网关VLAN</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>网关IP</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>备注信息</t>
         </is>
@@ -32245,22 +32236,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>己端设备</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>网关VLAN</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>网关IP</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>备注信息</t>
         </is>

</xml_diff>